<commit_message>
add WVS wave 7 reformulated questions
</commit_message>
<xml_diff>
--- a/data/WVS_Wave7_multiple_questions_selected_reformulated.xlsx
+++ b/data/WVS_Wave7_multiple_questions_selected_reformulated.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adeng/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adeng/Documents/py/MLLM-Joint-Publication/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312D4E11-19E0-7F48-8A57-F6EBDB27D28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D419AC2C-E4F1-784D-9F81-93A7D9201AA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10300" yWindow="4020" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="55">
   <si>
     <t>Code</t>
   </si>
@@ -162,17 +162,32 @@
     <t>Now we would like to know this respondent's opinion about the people from other countries who come to live in their country - the immigrants. How would this respondent evaluate the impact of these people on the development of their country?</t>
   </si>
   <si>
-    <t>Now I'd like to know this respondent's view on an issue. How would this respondent place their view on this scale? 1 means complete agreement with the statement on the left; 10 means complete agreement with the statement on the right; and if their views fall somewhere in between, any number in between is possible.</t>
-  </si>
-  <si>
     <t>How about people from other countries coming here to work. Which one of the following does this respondent think the government should do?</t>
-  </si>
-  <si>
-    <t>I'm going to describe a type of political system and ask what this respondent thinks about it as a way of governing this country. Would this respondent say it is a very good, fairly good, fairly bad or very bad way of governing this country? Having a strong leader who does not have to bother with parliament and elections.</t>
   </si>
   <si>
     <t xml:space="preserve"> 
 </t>
+  </si>
+  <si>
+    <t>For the following statement about the effects of immigration, does this respondent agree or disagree with it? Gives asylum to political refugees who are persecuted elsewhere.</t>
+  </si>
+  <si>
+    <t>1. Agree fully 2. Agree 3. Neither agree nor disagree 4. Disagree 5. Disagree fully</t>
+  </si>
+  <si>
+    <t>1. Fully agree 2. Agree 3. Disagree 4. Fully disagree</t>
+  </si>
+  <si>
+    <t>5. Highly beneficial 4. Beneficial 3. Neither beneficial nor detrimental 2. Detrimental 1. Highly detrimental</t>
+  </si>
+  <si>
+    <t>1. Highly beneficial 2. Beneficial 3. Detrimental 4. Highly detrimental</t>
+  </si>
+  <si>
+    <t>I'm going to describe a type of political system and ask what this respondent thinks about it as a way of governing this country. Would this respondent say it is a highly beneficial, beneficial, detrimental, or highly detrimental way of governing this country? Having a strong leader who does not have to bother with parliament and elections.</t>
+  </si>
+  <si>
+    <t>For the following statement, how strongly does this respondent agree or disagree with it? Does this respondent fully agree, agree, disagree, or fully disagree? When a mother works for pay, the children suffer.</t>
   </si>
 </sst>
 </file>
@@ -199,21 +214,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <strike/>
       <sz val="11"/>
       <color theme="1"/>
@@ -221,6 +221,19 @@
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -249,20 +262,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -571,137 +584,137 @@
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="92.33203125" customWidth="1"/>
-    <col min="3" max="3" width="77.33203125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="77.33203125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="60" x14ac:dyDescent="0.2">
+      <c r="C2" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="30" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="60" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="45" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="45" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="45" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="60" x14ac:dyDescent="0.2">
+      <c r="C7" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="45" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="64" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="45" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="64" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="63" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>30</v>
+      <c r="B11" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="B13" s="7" t="s">
-        <v>49</v>
+      <c r="B13" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="4" t="s">
         <v>44</v>
       </c>
     </row>

</xml_diff>